<commit_message>
Agrega histórico real de PMR para CR-L1032 (2013-2025)
Reemplaza la fila semilla de CR-L1032 en PMR_Historico.xlsx por los 13
ciclos reales aportados por el usuario (Segundo período enero-diciembre
2013 a 2025), incluyendo Estado del PMI e Indicador Sintético que la
semilla no tenía. El ciclo 2025 coincide con los valores de CPI(a)/SPI(a)/
Disb que ya traía la semilla, confirmando que corresponde al mismo ciclo
actual (I-2026).

Las demás 9 hojas quedan sin cambios, todavía con su fila semilla única.
</commit_message>
<xml_diff>
--- a/PMR_Historico.xlsx
+++ b/PMR_Historico.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -519,7 +519,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ciclo I-2026</t>
+          <t>Segundo período enero-diciembre 2025</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -541,14 +546,401 @@
       <c r="G4" t="n">
         <v>0.77</v>
       </c>
+      <c r="I4" t="n">
+        <v>2.2</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>ALERTA</t>
+          <t>Alerta</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>ALERTA</t>
+          <t>Alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2024</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.76</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2023</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.74</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2022</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2021</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.66</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Problema</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Problem</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2020</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.39</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.41</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2019</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1.01</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2018</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>0.49</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2017</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>SATISFACTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2016</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I13" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>SATISFACTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2015</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Problema</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>PROBLEM</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>SATISFACTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2013</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>SATISFACTORY</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega histórico real de PMR para CR-L1065 (2018-2025)
Reemplaza la fila semilla de CR-L1065 en PMR_Historico.xlsx por los 8
ciclos reales aportados por el usuario (Segundo período enero-diciembre
2018 a 2025). El ciclo 2025 coincide con los valores de CPI(a)/SPI(a)/Disb
que ya traía la semilla, confirmando que corresponde al ciclo actual
(I-2026). Este ciclo también trae el primer valor de T3 (6.00) del
histórico, coincidiendo con "Después del proyecto alcanza el 95% de los
desembolsos totales" como Estado del PMI.

Las demás 8 hojas quedan sin cambios, todavía con su fila semilla única.
</commit_message>
<xml_diff>
--- a/PMR_Historico.xlsx
+++ b/PMR_Historico.xlsx
@@ -1069,7 +1069,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1152,7 +1152,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ciclo I-2026</t>
+          <t>Segundo período enero-diciembre 2025</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Después del proyecto alcanza el 95% de los desembolsos totales</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1174,12 +1179,251 @@
       <c r="G4" t="n">
         <v>0.97</v>
       </c>
+      <c r="H4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>SATISFACTORIO</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2024</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.8100000000000001</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2023</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="I6" t="n">
+        <v>3</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2022</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1.11</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.64</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2021</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2020</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>1.17</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2019</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="n">
+        <v>7.94</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>SATISFACTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2018</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>3</v>
+      </c>
+      <c r="J11" t="inlineStr">
         <is>
           <t>SATISFACTORIO</t>
         </is>

</xml_diff>

<commit_message>
Agrega histórico real de PMR para CR-L1139 (2019-2025)
Reemplaza la fila semilla de CR-L1139 en PMR_Historico.xlsx por los 7
ciclos reales aportados por el usuario (Segundo período enero-diciembre
2019 a 2025). Para el ciclo 2025 se usan los valores de precisión completa
que ya traía la semilla (CPI/SPI/CPI(a)/SPI(a)/Disb), en vez de los
redondeados de la captura, ya que corresponden al mismo dato de origen.

Las demás 7 hojas quedan sin cambios, todavía con su fila semilla única.
</commit_message>
<xml_diff>
--- a/PMR_Historico.xlsx
+++ b/PMR_Historico.xlsx
@@ -1443,7 +1443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1526,7 +1526,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ciclo I-2026</t>
+          <t>Segundo período enero-diciembre 2025</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1544,6 +1549,9 @@
       <c r="G4" t="n">
         <v>0.6500000000000019</v>
       </c>
+      <c r="I4" t="n">
+        <v>2.85</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>SATISFACTORIO</t>
@@ -1551,7 +1559,224 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>SATISFACTORIO</t>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2024</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1.08</v>
+      </c>
+      <c r="D5" t="n">
+        <v>0.51</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2.85</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2023</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="D6" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.03</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.87</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.32</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2022</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="D7" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="E7" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.73</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.55</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2021</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1.04</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2020</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2019</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega histórico real de PMR para CR-L1151 (2023-2025)
Reemplaza la fila semilla de CR-L1151 en PMR_Historico.xlsx por los 3
ciclos reales aportados por el usuario (Segundo período enero-diciembre
2023 a 2025). El ciclo 2025 coincide exactamente con la semilla.

Las demás 6 hojas quedan sin cambios, todavía con su fila semilla única.
</commit_message>
<xml_diff>
--- a/PMR_Historico.xlsx
+++ b/PMR_Historico.xlsx
@@ -1794,7 +1794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1877,7 +1877,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ciclo I-2026</t>
+          <t>Segundo período enero-diciembre 2025</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1895,6 +1900,9 @@
       <c r="G4" t="n">
         <v>0.04</v>
       </c>
+      <c r="I4" t="n">
+        <v>2.9</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>SATISFACTORIO</t>
@@ -1902,7 +1910,49 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>SATISFACTORIO</t>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2024</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2023</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega histórico real de PMR para CR-L1137 (2019-2025)
Reemplaza la fila semilla de CR-L1137 en PMR_Historico.xlsx por los 7
ciclos reales aportados por el usuario (Segundo período enero-diciembre
2019 a 2025). El ciclo 2025 coincide exactamente con la semilla.

Las demás 5 hojas quedan sin cambios, todavía con su fila semilla única.
</commit_message>
<xml_diff>
--- a/PMR_Historico.xlsx
+++ b/PMR_Historico.xlsx
@@ -1970,7 +1970,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2053,7 +2053,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ciclo I-2026</t>
+          <t>Segundo período enero-diciembre 2025</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2075,14 +2080,197 @@
       <c r="G4" t="n">
         <v>0.65</v>
       </c>
+      <c r="I4" t="n">
+        <v>2.4</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>ALERTA</t>
+          <t>Alerta</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>SATISFACTORIO</t>
+          <t>SATISFACTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2024</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.97</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2023</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Alert</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2022</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2021</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="I8" t="n">
+        <v>3</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2020</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2019</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega histórico real de PMR para CR-J0002 (2023-2025)
3 ciclos según captura del usuario. Para el ciclo 2025 se usan los
valores de precisión completa que ya traía la semilla (CPI, SPI,
CPI(a), SPI(a), Disb) en vez de los redondeados de la imagen, dado
que corresponden al mismo dato subyacente.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NCVdRUSjtVxrCitHeuPnw8
</commit_message>
<xml_diff>
--- a/PMR_Historico.xlsx
+++ b/PMR_Historico.xlsx
@@ -2288,7 +2288,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2371,7 +2371,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ciclo I-2026</t>
+          <t>Segundo período enero-diciembre 2025</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -2389,14 +2394,79 @@
       <c r="G4" t="n">
         <v>0.3800000000000001</v>
       </c>
+      <c r="I4" t="n">
+        <v>1.8</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>PROBLEMA</t>
+          <t>Problema</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>PROBLEMA</t>
+          <t>Problem</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2024</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2023</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega histórico real de PMR para CR-L1066 (2015-2025)
11 ciclos según captura del usuario.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NCVdRUSjtVxrCitHeuPnw8
</commit_message>
<xml_diff>
--- a/PMR_Historico.xlsx
+++ b/PMR_Historico.xlsx
@@ -2484,7 +2484,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -2567,7 +2567,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ciclo I-2026</t>
+          <t>Segundo período enero-diciembre 2025</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Después del proyecto alcanza el 95% de los desembolsos totales</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -2589,6 +2594,12 @@
       <c r="G4" t="n">
         <v>1</v>
       </c>
+      <c r="H4" t="n">
+        <v>3</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
           <t>SATISFACTORIO</t>
@@ -2596,7 +2607,347 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>SATISFACTORIO</t>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2024</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="F5" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>SATISFACTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2023</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F6" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.7</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2022</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Alerta</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>SATISFACTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2021</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1.06</v>
+      </c>
+      <c r="F8" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Problema</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>ALERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2020</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="D9" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F9" t="n">
+        <v>1.16</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2.65</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2019</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="D10" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="E10" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0.84</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2018</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2017</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Después de la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" t="n">
+        <v>1</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>SATISFACTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2016</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>SATISFACTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2015</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>SATISFACTORY</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega histórico real de PMR para CR-L1152 (2024-2025)
2 ciclos según captura del usuario.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NCVdRUSjtVxrCitHeuPnw8
</commit_message>
<xml_diff>
--- a/PMR_Historico.xlsx
+++ b/PMR_Historico.xlsx
@@ -2965,7 +2965,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -3048,17 +3048,44 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ciclo I-2026</t>
+          <t>Segundo período enero-diciembre 2025</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>ALERTA</t>
+          <t>Alerta</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>SATISFACTORIO</t>
+          <t>SATISFACTORY</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Segundo período enero-diciembre 2024</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>SATISFACTORIO</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Satisfactory</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega histórico real de PMR para CR-L1157 (2025)
1 ciclo según captura del usuario (mismo dato que la semilla, solo
se ajusta la etiqueta de Ciclo y Estado del PMI).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NCVdRUSjtVxrCitHeuPnw8
</commit_message>
<xml_diff>
--- a/PMR_Historico.xlsx
+++ b/PMR_Historico.xlsx
@@ -1041,7 +1041,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Ciclo I-2026</t>
+          <t>Segundo período enero-diciembre 2025</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Desde la Aprobación hasta la Elegibilidad</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -1051,7 +1056,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>SATISFACTORIO</t>
+          <t>Satisfactory</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Traduce Clasificación Validada del histórico PMR a español
pmrPill() colorea las pills buscando las subcadenas en español
'SATISFACTORIO'/'ALERTA'/'PROBLEMA'. La columna Clasificación
Validada de PMR_Historico.xlsx tenía texto en inglés (Satisfactory/
Alert/Problem, en distintas variantes de mayúsculas) heredado de las
capturas originales, por lo que nunca matcheaba y la pill de
Validada siempre salía gris sin importar la calificación real.

Se traducen las 52 celdas afectadas (9 de las 10 hojas) a
Satisfactorio/Alerta/Problema. No se toca Clasificación Auto
calculada (ya estaba en español) ni ninguna otra columna.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NCVdRUSjtVxrCitHeuPnw8
</commit_message>
<xml_diff>
--- a/PMR_Historico.xlsx
+++ b/PMR_Historico.xlsx
@@ -556,7 +556,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Alerta</t>
         </is>
       </c>
     </row>
@@ -590,7 +590,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Alerta</t>
         </is>
       </c>
     </row>
@@ -624,7 +624,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Alerta</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Alerta</t>
         </is>
       </c>
     </row>
@@ -692,7 +692,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Problem</t>
+          <t>Problema</t>
         </is>
       </c>
     </row>
@@ -726,7 +726,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Alerta</t>
         </is>
       </c>
     </row>
@@ -760,7 +760,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Alerta</t>
         </is>
       </c>
     </row>
@@ -794,7 +794,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -834,7 +834,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -896,7 +896,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>PROBLEM</t>
+          <t>Problema</t>
         </is>
       </c>
     </row>
@@ -918,7 +918,7 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -940,7 +940,7 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1231,7 +1231,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1265,7 +1265,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1299,7 +1299,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1333,7 +1333,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1401,7 +1401,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1604,7 +1604,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1644,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1684,7 +1684,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1724,7 +1724,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1781,7 +1781,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -1957,7 +1957,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2095,7 +2095,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Alert</t>
+          <t>Alerta</t>
         </is>
       </c>
     </row>
@@ -2197,7 +2197,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2253,7 +2253,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2275,7 +2275,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2409,7 +2409,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Problem</t>
+          <t>Problema</t>
         </is>
       </c>
     </row>
@@ -2449,7 +2449,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2612,7 +2612,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2646,7 +2646,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2680,7 +2680,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2714,7 +2714,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2748,7 +2748,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>ALERT</t>
+          <t>Alerta</t>
         </is>
       </c>
     </row>
@@ -2788,7 +2788,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2868,7 +2868,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2908,7 +2908,7 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2930,7 +2930,7 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -2952,7 +2952,7 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -3068,7 +3068,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>SATISFACTORY</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Satisfactory</t>
+          <t>Satisfactorio</t>
         </is>
       </c>
     </row>

</xml_diff>